<commit_message>
Updated backend: added APScheduler and other changes
</commit_message>
<xml_diff>
--- a/backend/SuperTrend_Long.xlsx
+++ b/backend/SuperTrend_Long.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nanda\PycharmProjects\AlgoTrading\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AlgoTrading\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="73">
   <si>
     <t>Symbol</t>
   </si>
@@ -231,19 +231,13 @@
     <t>11-Apr-2025 11:40AM</t>
   </si>
   <si>
-    <t>11-Apr-2025 11:41AM</t>
-  </si>
-  <si>
-    <t>11-Apr-2025 12:14PM</t>
-  </si>
-  <si>
     <t>NIFTY 24 APR 2025 PE 23850.00</t>
   </si>
   <si>
-    <t>21-Apr-2025 10:45AM</t>
-  </si>
-  <si>
-    <t>21-Apr-2025 10:50AM</t>
+    <t>16-May-2025 10:45AM</t>
+  </si>
+  <si>
+    <t>16-May-2025 11:40AM</t>
   </si>
 </sst>
 </file>
@@ -608,6 +602,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:M45"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="27.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -1756,9 +1755,6 @@
       <c r="A31" t="s">
         <v>57</v>
       </c>
-      <c r="B31" t="s">
-        <v>69</v>
-      </c>
       <c r="C31">
         <v>116.3</v>
       </c>
@@ -2175,7 +2171,7 @@
         <v>57</v>
       </c>
       <c r="B42" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C42">
         <v>116.8</v>
@@ -2190,7 +2186,7 @@
         <v>75</v>
       </c>
       <c r="G42" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I42">
         <v>0</v>
@@ -2213,7 +2209,7 @@
         <v>57</v>
       </c>
       <c r="B43" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C43">
         <v>116.35</v>
@@ -2228,7 +2224,7 @@
         <v>75</v>
       </c>
       <c r="G43" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I43">
         <v>0.25</v>
@@ -2251,7 +2247,7 @@
         <v>57</v>
       </c>
       <c r="B44" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C44">
         <v>117.35</v>
@@ -2286,10 +2282,10 @@
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B45" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C45">
         <v>68.599999999999994</v>
@@ -2304,7 +2300,7 @@
         <v>75</v>
       </c>
       <c r="G45" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="I45">
         <v>-10.349999999999991</v>

</xml_diff>